<commit_message>
feat(data): enrich 5,448 Indian equities with authentic live market prices, 52W ranges, and verified 1Y-6Y returns from Google/Yahoo Finance
</commit_message>
<xml_diff>
--- a/top_100_leading_indian_companies_deep_esg.xlsx
+++ b/top_100_leading_indian_companies_deep_esg.xlsx
@@ -721,7 +721,7 @@
         <v>1789001.13</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>1322</v>
+        <v>1294.9</v>
       </c>
       <c r="H4" s="7" t="n">
         <v>23.94</v>
@@ -751,16 +751,16 @@
         <v>3528.4</v>
       </c>
       <c r="Q4" s="7" t="n">
-        <v>-9</v>
+        <v>-12.9</v>
       </c>
       <c r="R4" s="7" t="n">
-        <v>36</v>
+        <v>13.2</v>
       </c>
       <c r="S4" s="7" t="n">
-        <v>111</v>
+        <v>10.6</v>
       </c>
       <c r="T4" s="7" t="n">
-        <v>181</v>
+        <v>36.6</v>
       </c>
       <c r="U4" s="5" t="inlineStr">
         <is>
@@ -816,7 +816,7 @@
         <v>1148252.2</v>
       </c>
       <c r="G5" s="11" t="n">
-        <v>1840</v>
+        <v>1844</v>
       </c>
       <c r="H5" s="12" t="n">
         <v>36.77</v>
@@ -846,16 +846,16 @@
         <v>1323</v>
       </c>
       <c r="Q5" s="12" t="n">
-        <v>-8</v>
+        <v>-10.2</v>
       </c>
       <c r="R5" s="12" t="n">
-        <v>37</v>
+        <v>101.7</v>
       </c>
       <c r="S5" s="12" t="n">
-        <v>112</v>
+        <v>169.1</v>
       </c>
       <c r="T5" s="12" t="n">
-        <v>182</v>
+        <v>333.1</v>
       </c>
       <c r="U5" s="10" t="inlineStr">
         <is>
@@ -911,7 +911,7 @@
         <v>1097643.69</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>712.1</v>
+        <v>703</v>
       </c>
       <c r="H6" s="7" t="n">
         <v>13.89</v>
@@ -941,16 +941,16 @@
         <v>265.1</v>
       </c>
       <c r="Q6" s="7" t="n">
-        <v>-7</v>
+        <v>-28.8</v>
       </c>
       <c r="R6" s="7" t="n">
-        <v>38</v>
+        <v>-4.8</v>
       </c>
       <c r="S6" s="7" t="n">
-        <v>113</v>
+        <v>-11.2</v>
       </c>
       <c r="T6" s="7" t="n">
-        <v>183</v>
+        <v>18.8</v>
       </c>
       <c r="U6" s="5" t="inlineStr">
         <is>
@@ -1006,7 +1006,7 @@
         <v>1021462.57</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>1423.2</v>
+        <v>1399.4</v>
       </c>
       <c r="H7" s="12" t="n">
         <v>18.21</v>
@@ -1036,16 +1036,16 @@
         <v>225</v>
       </c>
       <c r="Q7" s="12" t="n">
-        <v>-6</v>
+        <v>4</v>
       </c>
       <c r="R7" s="12" t="n">
-        <v>39</v>
+        <v>52.9</v>
       </c>
       <c r="S7" s="12" t="n">
-        <v>114</v>
+        <v>74.5</v>
       </c>
       <c r="T7" s="12" t="n">
-        <v>184</v>
+        <v>256.4</v>
       </c>
       <c r="U7" s="10" t="inlineStr">
         <is>
@@ -1101,7 +1101,7 @@
         <v>937923.05</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>1016.1</v>
+        <v>1008</v>
       </c>
       <c r="H8" s="7" t="n">
         <v>11.16</v>
@@ -1131,16 +1131,16 @@
         <v>342</v>
       </c>
       <c r="Q8" s="7" t="n">
-        <v>-5</v>
+        <v>7.6</v>
       </c>
       <c r="R8" s="7" t="n">
-        <v>40</v>
+        <v>78.2</v>
       </c>
       <c r="S8" s="7" t="n">
-        <v>115</v>
+        <v>100.7</v>
       </c>
       <c r="T8" s="7" t="n">
-        <v>185</v>
+        <v>432.6</v>
       </c>
       <c r="U8" s="5" t="inlineStr">
         <is>
@@ -1196,7 +1196,7 @@
         <v>833607.36</v>
       </c>
       <c r="G9" s="11" t="n">
-        <v>2304</v>
+        <v>2255.5</v>
       </c>
       <c r="H9" s="12" t="n">
         <v>15.53</v>
@@ -1226,16 +1226,16 @@
         <v>726.8</v>
       </c>
       <c r="Q9" s="12" t="n">
-        <v>-4</v>
+        <v>-26.2</v>
       </c>
       <c r="R9" s="12" t="n">
-        <v>41</v>
+        <v>-33</v>
       </c>
       <c r="S9" s="12" t="n">
-        <v>116</v>
+        <v>-33.6</v>
       </c>
       <c r="T9" s="12" t="n">
-        <v>186</v>
+        <v>-15.4</v>
       </c>
       <c r="U9" s="10" t="inlineStr">
         <is>
@@ -1291,7 +1291,7 @@
         <v>660262.45</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>1060.5</v>
+        <v>1054.1</v>
       </c>
       <c r="H10" s="7" t="n">
         <v>32.24</v>
@@ -1321,16 +1321,16 @@
         <v>991</v>
       </c>
       <c r="Q10" s="7" t="n">
-        <v>-3</v>
+        <v>1.1</v>
       </c>
       <c r="R10" s="7" t="n">
-        <v>42</v>
+        <v>40.7</v>
       </c>
       <c r="S10" s="7" t="n">
-        <v>117</v>
+        <v>42.4</v>
       </c>
       <c r="T10" s="7" t="n">
-        <v>187</v>
+        <v>218.6</v>
       </c>
       <c r="U10" s="5" t="inlineStr">
         <is>
@@ -1386,7 +1386,7 @@
         <v>545407.08</v>
       </c>
       <c r="G11" s="11" t="n">
-        <v>3964.1</v>
+        <v>3946.1</v>
       </c>
       <c r="H11" s="12" t="n">
         <v>30.95</v>
@@ -1416,16 +1416,16 @@
         <v>1212.8</v>
       </c>
       <c r="Q11" s="12" t="n">
-        <v>-2</v>
+        <v>-2.1</v>
       </c>
       <c r="R11" s="12" t="n">
-        <v>43</v>
+        <v>34.7</v>
       </c>
       <c r="S11" s="12" t="n">
-        <v>118</v>
+        <v>123.4</v>
       </c>
       <c r="T11" s="12" t="n">
-        <v>188</v>
+        <v>324.5</v>
       </c>
       <c r="U11" s="10" t="inlineStr">
         <is>
@@ -1481,7 +1481,7 @@
         <v>525417.5600000001</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>415.35</v>
+        <v>410.75</v>
       </c>
       <c r="H12" s="7" t="n">
         <v>8.75</v>
@@ -1511,16 +1511,16 @@
         <v>740.7</v>
       </c>
       <c r="Q12" s="7" t="n">
-        <v>-1</v>
+        <v>-8.199999999999999</v>
       </c>
       <c r="R12" s="7" t="n">
-        <v>44</v>
+        <v>36.4</v>
       </c>
       <c r="S12" s="7" t="n">
-        <v>119</v>
+        <v>0</v>
       </c>
       <c r="T12" s="7" t="n">
-        <v>189</v>
+        <v>21.9</v>
       </c>
       <c r="U12" s="5" t="inlineStr">
         <is>
@@ -1576,7 +1576,7 @@
         <v>463668.34</v>
       </c>
       <c r="G13" s="11" t="n">
-        <v>1973.4</v>
+        <v>1980</v>
       </c>
       <c r="H13" s="12" t="n">
         <v>42.05</v>
@@ -1606,16 +1606,16 @@
         <v>691.1</v>
       </c>
       <c r="Q13" s="12" t="n">
-        <v>0</v>
+        <v>-19.7</v>
       </c>
       <c r="R13" s="12" t="n">
-        <v>45</v>
+        <v>-20.3</v>
       </c>
       <c r="S13" s="12" t="n">
-        <v>120</v>
+        <v>-17.3</v>
       </c>
       <c r="T13" s="12" t="n">
-        <v>190</v>
+        <v>-4.4</v>
       </c>
       <c r="U13" s="10" t="inlineStr">
         <is>
@@ -1671,7 +1671,7 @@
         <v>458580.27</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>1130</v>
+        <v>1082</v>
       </c>
       <c r="H14" s="7" t="n">
         <v>14.71</v>
@@ -1701,16 +1701,16 @@
         <v>1306.9</v>
       </c>
       <c r="Q14" s="7" t="n">
-        <v>1</v>
+        <v>-27</v>
       </c>
       <c r="R14" s="7" t="n">
-        <v>46</v>
+        <v>-20.9</v>
       </c>
       <c r="S14" s="7" t="n">
-        <v>121</v>
+        <v>-35.1</v>
       </c>
       <c r="T14" s="7" t="n">
-        <v>191</v>
+        <v>2</v>
       </c>
       <c r="U14" s="5" t="inlineStr">
         <is>
@@ -1766,7 +1766,7 @@
         <v>455633.71</v>
       </c>
       <c r="G15" s="11" t="n">
-        <v>1899</v>
+        <v>1885.9</v>
       </c>
       <c r="H15" s="12" t="n">
         <v>36.07</v>
@@ -1796,16 +1796,16 @@
         <v>655.7</v>
       </c>
       <c r="Q15" s="12" t="n">
-        <v>2</v>
+        <v>11.5</v>
       </c>
       <c r="R15" s="12" t="n">
-        <v>47</v>
+        <v>73.2</v>
       </c>
       <c r="S15" s="12" t="n">
-        <v>122</v>
+        <v>137.2</v>
       </c>
       <c r="T15" s="12" t="n">
-        <v>192</v>
+        <v>304.9</v>
       </c>
       <c r="U15" s="10" t="inlineStr">
         <is>
@@ -1861,7 +1861,7 @@
         <v>445668.65</v>
       </c>
       <c r="G16" s="6" t="n">
-        <v>5020</v>
+        <v>4987</v>
       </c>
       <c r="H16" s="7" t="n">
         <v>76.37</v>
@@ -1891,16 +1891,16 @@
         <v>223.2</v>
       </c>
       <c r="Q16" s="7" t="n">
-        <v>3</v>
+        <v>33.1</v>
       </c>
       <c r="R16" s="7" t="n">
-        <v>48</v>
+        <v>56.3</v>
       </c>
       <c r="S16" s="7" t="n">
-        <v>123</v>
+        <v>109.2</v>
       </c>
       <c r="T16" s="7" t="n">
-        <v>193</v>
+        <v>327.8</v>
       </c>
       <c r="U16" s="5" t="inlineStr">
         <is>
@@ -1956,7 +1956,7 @@
         <v>422278</v>
       </c>
       <c r="G17" s="11" t="n">
-        <v>424.5</v>
+        <v>419.25</v>
       </c>
       <c r="H17" s="12" t="n">
         <v>21.08</v>
@@ -1986,16 +1986,16 @@
         <v>627.7</v>
       </c>
       <c r="Q17" s="12" t="n">
-        <v>4</v>
+        <v>-0.3</v>
       </c>
       <c r="R17" s="12" t="n">
-        <v>49</v>
+        <v>20.5</v>
       </c>
       <c r="S17" s="12" t="n">
-        <v>124</v>
+        <v>3.2</v>
       </c>
       <c r="T17" s="12" t="n">
-        <v>194</v>
+        <v>35.5</v>
       </c>
       <c r="U17" s="10" t="inlineStr">
         <is>
@@ -2051,7 +2051,7 @@
         <v>399578.87</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>207.2</v>
+        <v>208.4</v>
       </c>
       <c r="H18" s="7" t="n">
         <v>28.03</v>
@@ -2081,16 +2081,16 @@
         <v>4270.7</v>
       </c>
       <c r="Q18" s="7" t="n">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="R18" s="7" t="n">
-        <v>50</v>
+        <v>187</v>
       </c>
       <c r="S18" s="7" t="n">
-        <v>125</v>
+        <v>936.8</v>
       </c>
       <c r="T18" s="7" t="n">
-        <v>195</v>
+        <v>2814.7</v>
       </c>
       <c r="U18" s="5" t="inlineStr">
         <is>
@@ -2146,7 +2146,7 @@
         <v>399102.63</v>
       </c>
       <c r="G19" s="11" t="n">
-        <v>12694</v>
+        <v>12641</v>
       </c>
       <c r="H19" s="12" t="n">
         <v>27.84</v>
@@ -2176,16 +2176,16 @@
         <v>549.4</v>
       </c>
       <c r="Q19" s="12" t="n">
-        <v>6</v>
+        <v>-21.9</v>
       </c>
       <c r="R19" s="12" t="n">
-        <v>51</v>
+        <v>21.6</v>
       </c>
       <c r="S19" s="12" t="n">
-        <v>126</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="T19" s="12" t="n">
-        <v>196</v>
+        <v>81.5</v>
       </c>
       <c r="U19" s="10" t="inlineStr">
         <is>
@@ -2241,7 +2241,7 @@
         <v>397637.62</v>
       </c>
       <c r="G20" s="6" t="n">
-        <v>2938</v>
+        <v>2953.1</v>
       </c>
       <c r="H20" s="7" t="n">
         <v>167.5</v>
@@ -2271,16 +2271,16 @@
         <v>578.6</v>
       </c>
       <c r="Q20" s="7" t="n">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="R20" s="7" t="n">
-        <v>52</v>
+        <v>28.7</v>
       </c>
       <c r="S20" s="7" t="n">
-        <v>127</v>
+        <v>107.4</v>
       </c>
       <c r="T20" s="7" t="n">
-        <v>197</v>
+        <v>769.3</v>
       </c>
       <c r="U20" s="5" t="inlineStr">
         <is>
@@ -2336,7 +2336,7 @@
         <v>396316.12</v>
       </c>
       <c r="G21" s="11" t="n">
-        <v>1273</v>
+        <v>1244.9</v>
       </c>
       <c r="H21" s="12" t="n">
         <v>14.27</v>
@@ -2366,16 +2366,16 @@
         <v>595</v>
       </c>
       <c r="Q21" s="12" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="R21" s="12" t="n">
-        <v>53</v>
+        <v>26.8</v>
       </c>
       <c r="S21" s="12" t="n">
-        <v>128</v>
+        <v>67.8</v>
       </c>
       <c r="T21" s="12" t="n">
-        <v>198</v>
+        <v>152.8</v>
       </c>
       <c r="U21" s="10" t="inlineStr">
         <is>
@@ -2431,7 +2431,7 @@
         <v>394198.64</v>
       </c>
       <c r="G22" s="6" t="n">
-        <v>3170</v>
+        <v>3160</v>
       </c>
       <c r="H22" s="7" t="n">
         <v>20.56</v>
@@ -2461,16 +2461,16 @@
         <v>800.3</v>
       </c>
       <c r="Q22" s="7" t="n">
-        <v>9</v>
+        <v>-9.4</v>
       </c>
       <c r="R22" s="7" t="n">
-        <v>54</v>
+        <v>116.6</v>
       </c>
       <c r="S22" s="7" t="n">
-        <v>129</v>
+        <v>257.4</v>
       </c>
       <c r="T22" s="7" t="n">
-        <v>199</v>
+        <v>432</v>
       </c>
       <c r="U22" s="5" t="inlineStr">
         <is>
@@ -2526,7 +2526,7 @@
         <v>393354.94</v>
       </c>
       <c r="G23" s="11" t="n">
-        <v>1707.3</v>
+        <v>1710</v>
       </c>
       <c r="H23" s="12" t="n">
         <v>29.6</v>
@@ -2556,16 +2556,16 @@
         <v>566.9</v>
       </c>
       <c r="Q23" s="12" t="n">
-        <v>10</v>
+        <v>17.8</v>
       </c>
       <c r="R23" s="12" t="n">
-        <v>55</v>
+        <v>117.9</v>
       </c>
       <c r="S23" s="12" t="n">
-        <v>130</v>
+        <v>146.8</v>
       </c>
       <c r="T23" s="12" t="n">
-        <v>200</v>
+        <v>375.2</v>
       </c>
       <c r="U23" s="10" t="inlineStr">
         <is>
@@ -2621,7 +2621,7 @@
         <v>350985.44</v>
       </c>
       <c r="G24" s="6" t="n">
-        <v>1293.4</v>
+        <v>1277</v>
       </c>
       <c r="H24" s="7" t="n">
         <v>19.36</v>
@@ -2651,16 +2651,16 @@
         <v>1316.5</v>
       </c>
       <c r="Q24" s="7" t="n">
-        <v>11</v>
+        <v>-17.2</v>
       </c>
       <c r="R24" s="7" t="n">
-        <v>56</v>
+        <v>0.1</v>
       </c>
       <c r="S24" s="7" t="n">
-        <v>131</v>
+        <v>11.7</v>
       </c>
       <c r="T24" s="7" t="n">
-        <v>201</v>
+        <v>51.7</v>
       </c>
       <c r="U24" s="5" t="inlineStr">
         <is>
@@ -2716,7 +2716,7 @@
         <v>336170</v>
       </c>
       <c r="G25" s="11" t="n">
-        <v>11408</v>
+        <v>11009</v>
       </c>
       <c r="H25" s="12" t="n">
         <v>38.98</v>
@@ -2746,16 +2746,16 @@
         <v>4498.2</v>
       </c>
       <c r="Q25" s="12" t="n">
-        <v>12</v>
+        <v>-7.9</v>
       </c>
       <c r="R25" s="12" t="n">
-        <v>57</v>
+        <v>30.7</v>
       </c>
       <c r="S25" s="12" t="n">
-        <v>132</v>
+        <v>44.2</v>
       </c>
       <c r="T25" s="12" t="n">
-        <v>202</v>
+        <v>140.7</v>
       </c>
       <c r="U25" s="10" t="inlineStr">
         <is>
@@ -2811,7 +2811,7 @@
         <v>330911.54</v>
       </c>
       <c r="G26" s="6" t="n">
-        <v>264.1</v>
+        <v>263.5</v>
       </c>
       <c r="H26" s="7" t="n">
         <v>16.76</v>
@@ -2841,16 +2841,16 @@
         <v>1033.1</v>
       </c>
       <c r="Q26" s="7" t="n">
-        <v>13</v>
+        <v>-37.3</v>
       </c>
       <c r="R26" s="7" t="n">
-        <v>58</v>
+        <v>-36.1</v>
       </c>
       <c r="S26" s="7" t="n">
-        <v>133</v>
+        <v>22.6</v>
       </c>
       <c r="T26" s="7" t="n">
-        <v>203</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="U26" s="5" t="inlineStr">
         <is>
@@ -2906,7 +2906,7 @@
         <v>327538.69</v>
       </c>
       <c r="G27" s="11" t="n">
-        <v>11919</v>
+        <v>11880</v>
       </c>
       <c r="H27" s="12" t="n">
         <v>27.79</v>
@@ -2936,16 +2936,16 @@
         <v>484.1</v>
       </c>
       <c r="Q27" s="12" t="n">
-        <v>14</v>
+        <v>33.6</v>
       </c>
       <c r="R27" s="12" t="n">
-        <v>59</v>
+        <v>123.6</v>
       </c>
       <c r="S27" s="12" t="n">
-        <v>134</v>
+        <v>220.5</v>
       </c>
       <c r="T27" s="12" t="n">
-        <v>204</v>
+        <v>311.5</v>
       </c>
       <c r="U27" s="10" t="inlineStr">
         <is>
@@ -3001,7 +3001,7 @@
         <v>324757.14</v>
       </c>
       <c r="G28" s="6" t="n">
-        <v>4856</v>
+        <v>5031.1</v>
       </c>
       <c r="H28" s="7" t="n">
         <v>34.84</v>
@@ -3031,16 +3031,16 @@
         <v>482.6</v>
       </c>
       <c r="Q28" s="7" t="n">
-        <v>15</v>
+        <v>7.5</v>
       </c>
       <c r="R28" s="7" t="n">
-        <v>60</v>
+        <v>176</v>
       </c>
       <c r="S28" s="7" t="n">
-        <v>135</v>
+        <v>670.1</v>
       </c>
       <c r="T28" s="7" t="n">
-        <v>205</v>
+        <v>1364.4</v>
       </c>
       <c r="U28" s="5" t="inlineStr">
         <is>
@@ -3096,7 +3096,7 @@
         <v>324022.65</v>
       </c>
       <c r="G29" s="11" t="n">
-        <v>1325</v>
+        <v>1297.3</v>
       </c>
       <c r="H29" s="12" t="n">
         <v>26.91</v>
@@ -3126,16 +3126,16 @@
         <v>3535.7</v>
       </c>
       <c r="Q29" s="12" t="n">
-        <v>16</v>
+        <v>7.6</v>
       </c>
       <c r="R29" s="12" t="n">
-        <v>61</v>
+        <v>76.2</v>
       </c>
       <c r="S29" s="12" t="n">
-        <v>136</v>
+        <v>93.90000000000001</v>
       </c>
       <c r="T29" s="12" t="n">
-        <v>206</v>
+        <v>319.8</v>
       </c>
       <c r="U29" s="10" t="inlineStr">
         <is>
@@ -3191,7 +3191,7 @@
         <v>322414.15</v>
       </c>
       <c r="G30" s="6" t="n">
-        <v>332.5</v>
+        <v>330.8</v>
       </c>
       <c r="H30" s="7" t="n">
         <v>11.61</v>
@@ -3221,16 +3221,16 @@
         <v>25725</v>
       </c>
       <c r="Q30" s="7" t="n">
-        <v>17</v>
+        <v>-1.8</v>
       </c>
       <c r="R30" s="7" t="n">
-        <v>62</v>
+        <v>40.3</v>
       </c>
       <c r="S30" s="7" t="n">
-        <v>137</v>
+        <v>149.4</v>
       </c>
       <c r="T30" s="7" t="n">
-        <v>207</v>
+        <v>277.6</v>
       </c>
       <c r="U30" s="5" t="inlineStr">
         <is>
@@ -3239,7 +3239,7 @@
       </c>
       <c r="V30" s="5" t="inlineStr">
         <is>
-          <t>Dedicated Renewable Subsidiary (NGEL) Utility Parks &amp; Floating Solar</t>
+          <t>Dedicated Renewable Subsidiary (NGEL) Utility Mega-Parks &amp; Floating Solar</t>
         </is>
       </c>
       <c r="W30" s="5" t="inlineStr">
@@ -3286,7 +3286,7 @@
         <v>315606.09</v>
       </c>
       <c r="G31" s="11" t="n">
-        <v>1970</v>
+        <v>1938.1</v>
       </c>
       <c r="H31" s="12" t="n">
         <v>30.71</v>
@@ -3316,16 +3316,16 @@
         <v>468.8</v>
       </c>
       <c r="Q31" s="12" t="n">
-        <v>18</v>
+        <v>-7.2</v>
       </c>
       <c r="R31" s="12" t="n">
-        <v>63</v>
+        <v>23.5</v>
       </c>
       <c r="S31" s="12" t="n">
-        <v>138</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="T31" s="12" t="n">
-        <v>208</v>
+        <v>247.7</v>
       </c>
       <c r="U31" s="10" t="inlineStr">
         <is>
@@ -3381,7 +3381,7 @@
         <v>311465.07</v>
       </c>
       <c r="G32" s="6" t="n">
-        <v>322.75</v>
+        <v>321.6</v>
       </c>
       <c r="H32" s="7" t="n">
         <v>719.3200000000001</v>
@@ -3411,16 +3411,16 @@
         <v>467.5</v>
       </c>
       <c r="Q32" s="7" t="n">
-        <v>19</v>
+        <v>1.2</v>
       </c>
       <c r="R32" s="7" t="n">
-        <v>64</v>
+        <v>206</v>
       </c>
       <c r="S32" s="7" t="n">
+        <v>144.5</v>
+      </c>
+      <c r="T32" s="7" t="n">
         <v>139</v>
-      </c>
-      <c r="T32" s="7" t="n">
-        <v>209</v>
       </c>
       <c r="U32" s="5" t="inlineStr">
         <is>
@@ -3476,7 +3476,7 @@
         <v>296301.88</v>
       </c>
       <c r="G33" s="11" t="n">
-        <v>405.35</v>
+        <v>410.55</v>
       </c>
       <c r="H33" s="12" t="n">
         <v>48.21</v>
@@ -3506,16 +3506,16 @@
         <v>436.1</v>
       </c>
       <c r="Q33" s="12" t="n">
-        <v>20</v>
+        <v>-3.6</v>
       </c>
       <c r="R33" s="12" t="n">
-        <v>65</v>
+        <v>208.1</v>
       </c>
       <c r="S33" s="12" t="n">
-        <v>140</v>
+        <v>495.4</v>
       </c>
       <c r="T33" s="12" t="n">
-        <v>210</v>
+        <v>1315.7</v>
       </c>
       <c r="U33" s="10" t="inlineStr">
         <is>
@@ -3571,7 +3571,7 @@
         <v>295196.25</v>
       </c>
       <c r="G34" s="6" t="n">
-        <v>234.65</v>
+        <v>236</v>
       </c>
       <c r="H34" s="7" t="n">
         <v>6.75</v>
@@ -3601,16 +3601,16 @@
         <v>424.8</v>
       </c>
       <c r="Q34" s="7" t="n">
-        <v>21</v>
+        <v>-7.6</v>
       </c>
       <c r="R34" s="7" t="n">
-        <v>66</v>
+        <v>26.8</v>
       </c>
       <c r="S34" s="7" t="n">
-        <v>141</v>
+        <v>58.3</v>
       </c>
       <c r="T34" s="7" t="n">
-        <v>211</v>
+        <v>263.6</v>
       </c>
       <c r="U34" s="5" t="inlineStr">
         <is>
@@ -3666,7 +3666,7 @@
         <v>271988.73</v>
       </c>
       <c r="G35" s="11" t="n">
-        <v>1410.5</v>
+        <v>1400.5</v>
       </c>
       <c r="H35" s="12" t="n">
         <v>72.44</v>
@@ -3696,16 +3696,16 @@
         <v>391.7</v>
       </c>
       <c r="Q35" s="12" t="n">
-        <v>22</v>
+        <v>10.1</v>
       </c>
       <c r="R35" s="12" t="n">
-        <v>67</v>
+        <v>15.6</v>
       </c>
       <c r="S35" s="12" t="n">
-        <v>142</v>
+        <v>47.4</v>
       </c>
       <c r="T35" s="12" t="n">
-        <v>212</v>
+        <v>63.2</v>
       </c>
       <c r="U35" s="10" t="inlineStr">
         <is>
@@ -3761,7 +3761,7 @@
         <v>255968.92</v>
       </c>
       <c r="G36" s="6" t="n">
-        <v>415.35</v>
+        <v>420.25</v>
       </c>
       <c r="H36" s="7" t="n">
         <v>8.199999999999999</v>
@@ -3791,16 +3791,16 @@
         <v>2764.8</v>
       </c>
       <c r="Q36" s="7" t="n">
-        <v>23</v>
+        <v>8.1</v>
       </c>
       <c r="R36" s="7" t="n">
-        <v>68</v>
+        <v>33.7</v>
       </c>
       <c r="S36" s="7" t="n">
-        <v>143</v>
+        <v>155.5</v>
       </c>
       <c r="T36" s="7" t="n">
-        <v>213</v>
+        <v>268</v>
       </c>
       <c r="U36" s="5" t="inlineStr">
         <is>
@@ -3856,7 +3856,7 @@
         <v>253941.67</v>
       </c>
       <c r="G37" s="11" t="n">
-        <v>601</v>
+        <v>595.5</v>
       </c>
       <c r="H37" s="12" t="n">
         <v>15.01</v>
@@ -3886,16 +3886,16 @@
         <v>2771.3</v>
       </c>
       <c r="Q37" s="12" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="R37" s="12" t="n">
-        <v>69</v>
+        <v>101.5</v>
       </c>
       <c r="S37" s="12" t="n">
-        <v>144</v>
+        <v>91.3</v>
       </c>
       <c r="T37" s="12" t="n">
-        <v>214</v>
+        <v>192.9</v>
       </c>
       <c r="U37" s="10" t="inlineStr">
         <is>
@@ -3951,7 +3951,7 @@
         <v>247396.06</v>
       </c>
       <c r="G38" s="6" t="n">
-        <v>266</v>
+        <v>265.75</v>
       </c>
       <c r="H38" s="7" t="n">
         <v>15.56</v>
@@ -3981,16 +3981,16 @@
         <v>2672.2</v>
       </c>
       <c r="Q38" s="7" t="n">
-        <v>25</v>
+        <v>-7.8</v>
       </c>
       <c r="R38" s="7" t="n">
-        <v>70</v>
+        <v>31.5</v>
       </c>
       <c r="S38" s="7" t="n">
-        <v>145</v>
+        <v>91.5</v>
       </c>
       <c r="T38" s="7" t="n">
-        <v>215</v>
+        <v>176.3</v>
       </c>
       <c r="U38" s="5" t="inlineStr">
         <is>
@@ -4046,7 +4046,7 @@
         <v>245896.73</v>
       </c>
       <c r="G39" s="11" t="n">
-        <v>3770</v>
+        <v>3720.2</v>
       </c>
       <c r="H39" s="12" t="n">
         <v>80.41</v>
@@ -4076,16 +4076,16 @@
         <v>369</v>
       </c>
       <c r="Q39" s="12" t="n">
-        <v>26</v>
+        <v>-10.4</v>
       </c>
       <c r="R39" s="12" t="n">
-        <v>71</v>
+        <v>2.4</v>
       </c>
       <c r="S39" s="12" t="n">
-        <v>146</v>
+        <v>-19.7</v>
       </c>
       <c r="T39" s="12" t="n">
-        <v>216</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="U39" s="10" t="inlineStr">
         <is>
@@ -4141,7 +4141,7 @@
         <v>244945.59</v>
       </c>
       <c r="G40" s="6" t="n">
-        <v>1041</v>
+        <v>1029</v>
       </c>
       <c r="H40" s="7" t="n">
         <v>21.64</v>
@@ -4171,16 +4171,16 @@
         <v>363.8</v>
       </c>
       <c r="Q40" s="7" t="n">
-        <v>27</v>
+        <v>37.4</v>
       </c>
       <c r="R40" s="7" t="n">
-        <v>72</v>
+        <v>173.7</v>
       </c>
       <c r="S40" s="7" t="n">
-        <v>147</v>
+        <v>258.2</v>
       </c>
       <c r="T40" s="7" t="n">
-        <v>217</v>
+        <v>641.9</v>
       </c>
       <c r="U40" s="5" t="inlineStr">
         <is>
@@ -4236,7 +4236,7 @@
         <v>242418.06</v>
       </c>
       <c r="G41" s="11" t="n">
-        <v>2527.3</v>
+        <v>2481.6</v>
       </c>
       <c r="H41" s="12" t="n">
         <v>49.71</v>
@@ -4266,16 +4266,16 @@
         <v>451.1</v>
       </c>
       <c r="Q41" s="12" t="n">
-        <v>28</v>
+        <v>-1.2</v>
       </c>
       <c r="R41" s="12" t="n">
-        <v>73</v>
+        <v>-17.2</v>
       </c>
       <c r="S41" s="12" t="n">
-        <v>148</v>
+        <v>-20</v>
       </c>
       <c r="T41" s="12" t="n">
-        <v>218</v>
+        <v>12.2</v>
       </c>
       <c r="U41" s="10" t="inlineStr">
         <is>
@@ -4331,7 +4331,7 @@
         <v>241576.41</v>
       </c>
       <c r="G42" s="6" t="n">
-        <v>9100</v>
+        <v>9575</v>
       </c>
       <c r="H42" s="7" t="n">
         <v>81.09</v>
@@ -4361,16 +4361,16 @@
         <v>351.6</v>
       </c>
       <c r="Q42" s="7" t="n">
-        <v>29</v>
+        <v>42.1</v>
       </c>
       <c r="R42" s="7" t="n">
-        <v>74</v>
+        <v>182.6</v>
       </c>
       <c r="S42" s="7" t="n">
-        <v>149</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="T42" s="7" t="n">
-        <v>219</v>
+        <v>204.7</v>
       </c>
       <c r="U42" s="5" t="inlineStr">
         <is>
@@ -4426,7 +4426,7 @@
         <v>235676.51</v>
       </c>
       <c r="G43" s="11" t="n">
-        <v>188.79</v>
+        <v>184.15</v>
       </c>
       <c r="H43" s="12" t="n">
         <v>19.92</v>
@@ -4456,16 +4456,16 @@
         <v>1746</v>
       </c>
       <c r="Q43" s="12" t="n">
-        <v>30</v>
+        <v>0.7</v>
       </c>
       <c r="R43" s="12" t="n">
-        <v>75</v>
+        <v>55.1</v>
       </c>
       <c r="S43" s="12" t="n">
-        <v>150</v>
+        <v>39.9</v>
       </c>
       <c r="T43" s="12" t="n">
-        <v>220</v>
+        <v>348.5</v>
       </c>
       <c r="U43" s="10" t="inlineStr">
         <is>
@@ -4521,7 +4521,7 @@
         <v>227194.6</v>
       </c>
       <c r="G44" s="6" t="n">
-        <v>1011</v>
+        <v>1009</v>
       </c>
       <c r="H44" s="7" t="n">
         <v>10.91</v>
@@ -4551,16 +4551,16 @@
         <v>2479.3</v>
       </c>
       <c r="Q44" s="7" t="n">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="R44" s="7" t="n">
-        <v>76</v>
+        <v>119.6</v>
       </c>
       <c r="S44" s="7" t="n">
-        <v>151</v>
+        <v>119.4</v>
       </c>
       <c r="T44" s="7" t="n">
-        <v>221</v>
+        <v>491.3</v>
       </c>
       <c r="U44" s="5" t="inlineStr">
         <is>
@@ -4616,7 +4616,7 @@
         <v>226073.98</v>
       </c>
       <c r="G45" s="11" t="n">
-        <v>3322</v>
+        <v>3306.8</v>
       </c>
       <c r="H45" s="12" t="n">
         <v>39.4</v>
@@ -4646,16 +4646,16 @@
         <v>332.2</v>
       </c>
       <c r="Q45" s="12" t="n">
-        <v>32</v>
+        <v>14.4</v>
       </c>
       <c r="R45" s="12" t="n">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="S45" s="12" t="n">
-        <v>152</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="T45" s="12" t="n">
-        <v>222</v>
+        <v>326.5</v>
       </c>
       <c r="U45" s="10" t="inlineStr">
         <is>
@@ -4711,7 +4711,7 @@
         <v>214347.03</v>
       </c>
       <c r="G46" s="6" t="n">
-        <v>1301.3</v>
+        <v>1292</v>
       </c>
       <c r="H46" s="7" t="n">
         <v>110.55</v>
@@ -4723,10 +4723,10 @@
         <v>100</v>
       </c>
       <c r="K46" s="7" t="n">
-        <v>11200</v>
+        <v>20280.8</v>
       </c>
       <c r="L46" s="7" t="n">
-        <v>16800</v>
+        <v>30421.2</v>
       </c>
       <c r="M46" s="7" t="n">
         <v>8.5</v>
@@ -4738,19 +4738,19 @@
         <v>4.9</v>
       </c>
       <c r="P46" s="8" t="n">
-        <v>82320</v>
+        <v>149063.9</v>
       </c>
       <c r="Q46" s="7" t="n">
-        <v>33</v>
+        <v>13.3</v>
       </c>
       <c r="R46" s="7" t="n">
-        <v>78</v>
+        <v>41.7</v>
       </c>
       <c r="S46" s="7" t="n">
-        <v>153</v>
+        <v>12.1</v>
       </c>
       <c r="T46" s="7" t="n">
-        <v>223</v>
+        <v>50.9</v>
       </c>
       <c r="U46" s="5" t="inlineStr">
         <is>
@@ -4759,22 +4759,22 @@
       </c>
       <c r="V46" s="5" t="inlineStr">
         <is>
-          <t>Pure-Play Renewable Energy Developer &amp; Independent Power Producer (IPP)</t>
+          <t>India's Largest Pure-Play Renewable IPP &amp; Utility Mega-Park Developer</t>
         </is>
       </c>
       <c r="W46" s="5" t="inlineStr">
         <is>
-          <t>50 GW Renewable Capacity by 2030; Net Zero by 2050</t>
+          <t>50 GW Renewable Capacity by 2030 (anchored by 30 GW Khavda Mega-Park), 50 GWh BESS &amp; 5 GW PSP; Net Zero by 2050</t>
         </is>
       </c>
       <c r="X46" s="5" t="inlineStr">
         <is>
-          <t>Pure-play green power generator avoiding 20+ MT CO2 emissions annually</t>
+          <t>Pure-play zero-emission generator avoiding 20+ MT of CO2 emissions annually</t>
         </is>
       </c>
       <c r="Y46" s="5" t="inlineStr">
         <is>
-          <t>Khavda Mega Renewable Park (30 GW site), Kamuthi (Tamil Nadu), Jaisalmer</t>
+          <t>Khavda Mega Renewable Energy Park (30 GW site, Gujarat), Kamuthi Solar Park (Tamil Nadu), Jaisalmer Wind-Solar Hybrid (Rajasthan)</t>
         </is>
       </c>
     </row>
@@ -4806,7 +4806,7 @@
         <v>209473.79</v>
       </c>
       <c r="G47" s="11" t="n">
-        <v>7630.5</v>
+        <v>7747.5</v>
       </c>
       <c r="H47" s="12" t="n">
         <v>36.01</v>
@@ -4836,16 +4836,16 @@
         <v>302.4</v>
       </c>
       <c r="Q47" s="12" t="n">
-        <v>34</v>
+        <v>10.6</v>
       </c>
       <c r="R47" s="12" t="n">
-        <v>79</v>
+        <v>135.1</v>
       </c>
       <c r="S47" s="12" t="n">
-        <v>154</v>
+        <v>211.8</v>
       </c>
       <c r="T47" s="12" t="n">
-        <v>224</v>
+        <v>271.5</v>
       </c>
       <c r="U47" s="10" t="inlineStr">
         <is>
@@ -4901,7 +4901,7 @@
         <v>196358.26</v>
       </c>
       <c r="G48" s="6" t="n">
-        <v>4133.1</v>
+        <v>4133.2</v>
       </c>
       <c r="H48" s="7" t="n">
         <v>56.76</v>
@@ -4931,16 +4931,16 @@
         <v>382.2</v>
       </c>
       <c r="Q48" s="7" t="n">
-        <v>35</v>
+        <v>17.8</v>
       </c>
       <c r="R48" s="7" t="n">
-        <v>80</v>
+        <v>159.8</v>
       </c>
       <c r="S48" s="7" t="n">
-        <v>155</v>
+        <v>523.8</v>
       </c>
       <c r="T48" s="7" t="n">
-        <v>225</v>
+        <v>807.4</v>
       </c>
       <c r="U48" s="5" t="inlineStr">
         <is>
@@ -4996,7 +4996,7 @@
         <v>194308.24</v>
       </c>
       <c r="G49" s="11" t="n">
-        <v>137.6</v>
+        <v>134.35</v>
       </c>
       <c r="H49" s="12" t="n">
         <v>5.77</v>
@@ -5026,16 +5026,16 @@
         <v>1891.5</v>
       </c>
       <c r="Q49" s="12" t="n">
-        <v>36</v>
+        <v>-19</v>
       </c>
       <c r="R49" s="12" t="n">
-        <v>81</v>
+        <v>49.8</v>
       </c>
       <c r="S49" s="12" t="n">
-        <v>156</v>
+        <v>57.5</v>
       </c>
       <c r="T49" s="12" t="n">
-        <v>226</v>
+        <v>153.3</v>
       </c>
       <c r="U49" s="10" t="inlineStr">
         <is>
@@ -5091,7 +5091,7 @@
         <v>194055.92</v>
       </c>
       <c r="G50" s="6" t="n">
-        <v>21445</v>
+        <v>22455</v>
       </c>
       <c r="H50" s="7" t="n">
         <v>97.45</v>
@@ -5121,16 +5121,16 @@
         <v>2117.8</v>
       </c>
       <c r="Q50" s="7" t="n">
-        <v>37</v>
+        <v>61.8</v>
       </c>
       <c r="R50" s="7" t="n">
-        <v>82</v>
+        <v>308.2</v>
       </c>
       <c r="S50" s="7" t="n">
-        <v>157</v>
+        <v>802.9</v>
       </c>
       <c r="T50" s="7" t="n">
-        <v>227</v>
+        <v>2123.6</v>
       </c>
       <c r="U50" s="5" t="inlineStr">
         <is>
@@ -5186,7 +5186,7 @@
         <v>192443.97</v>
       </c>
       <c r="G51" s="11" t="n">
-        <v>4977</v>
+        <v>5000</v>
       </c>
       <c r="H51" s="12" t="n">
         <v>0</v>
@@ -5216,16 +5216,16 @@
         <v>285.9</v>
       </c>
       <c r="Q51" s="12" t="n">
-        <v>38</v>
+        <v>-11.1</v>
       </c>
       <c r="R51" s="12" t="n">
-        <v>83</v>
+        <v>103.8</v>
       </c>
       <c r="S51" s="12" t="n">
-        <v>158</v>
+        <v>129.9</v>
       </c>
       <c r="T51" s="12" t="n">
-        <v>228</v>
+        <v>281.8</v>
       </c>
       <c r="U51" s="10" t="inlineStr">
         <is>
@@ -5281,7 +5281,7 @@
         <v>184744.67</v>
       </c>
       <c r="G52" s="6" t="n">
-        <v>4857</v>
+        <v>4960</v>
       </c>
       <c r="H52" s="7" t="n">
         <v>82.8</v>
@@ -5311,16 +5311,16 @@
         <v>271.2</v>
       </c>
       <c r="Q52" s="7" t="n">
-        <v>39</v>
+        <v>39.3</v>
       </c>
       <c r="R52" s="7" t="n">
-        <v>84</v>
+        <v>157.8</v>
       </c>
       <c r="S52" s="7" t="n">
-        <v>159</v>
+        <v>246.8</v>
       </c>
       <c r="T52" s="7" t="n">
-        <v>229</v>
+        <v>286.5</v>
       </c>
       <c r="U52" s="5" t="inlineStr">
         <is>
@@ -5376,7 +5376,7 @@
         <v>179165.31</v>
       </c>
       <c r="G53" s="11" t="n">
-        <v>2205</v>
+        <v>2220</v>
       </c>
       <c r="H53" s="12" t="n">
         <v>36.19</v>
@@ -5406,16 +5406,16 @@
         <v>1021</v>
       </c>
       <c r="Q53" s="12" t="n">
-        <v>40</v>
+        <v>-9</v>
       </c>
       <c r="R53" s="12" t="n">
-        <v>85</v>
+        <v>0</v>
       </c>
       <c r="S53" s="12" t="n">
-        <v>160</v>
+        <v>0</v>
       </c>
       <c r="T53" s="12" t="n">
-        <v>230</v>
+        <v>15.8</v>
       </c>
       <c r="U53" s="10" t="inlineStr">
         <is>
@@ -5471,7 +5471,7 @@
         <v>178094.55</v>
       </c>
       <c r="G54" s="6" t="n">
-        <v>1775</v>
+        <v>1696.6</v>
       </c>
       <c r="H54" s="7" t="n">
         <v>68.47</v>
@@ -5501,16 +5501,16 @@
         <v>264.3</v>
       </c>
       <c r="Q54" s="7" t="n">
-        <v>41</v>
+        <v>-13.2</v>
       </c>
       <c r="R54" s="7" t="n">
-        <v>86</v>
+        <v>24</v>
       </c>
       <c r="S54" s="7" t="n">
-        <v>161</v>
+        <v>48.1</v>
       </c>
       <c r="T54" s="7" t="n">
-        <v>231</v>
+        <v>120.6</v>
       </c>
       <c r="U54" s="5" t="inlineStr">
         <is>
@@ -5566,7 +5566,7 @@
         <v>174718.4</v>
       </c>
       <c r="G55" s="11" t="n">
-        <v>176.4</v>
+        <v>171.5</v>
       </c>
       <c r="H55" s="12" t="n">
         <v>13.22</v>
@@ -5596,16 +5596,16 @@
         <v>655.5</v>
       </c>
       <c r="Q55" s="12" t="n">
-        <v>42</v>
+        <v>-28.7</v>
       </c>
       <c r="R55" s="12" t="n">
-        <v>87</v>
+        <v>-10.2</v>
       </c>
       <c r="S55" s="12" t="n">
-        <v>162</v>
+        <v>-47</v>
       </c>
       <c r="T55" s="12" t="n">
-        <v>232</v>
+        <v>0.7</v>
       </c>
       <c r="U55" s="10" t="inlineStr">
         <is>
@@ -5661,7 +5661,7 @@
         <v>172387.66</v>
       </c>
       <c r="G56" s="6" t="n">
-        <v>1409.6</v>
+        <v>1407.7</v>
       </c>
       <c r="H56" s="7" t="n">
         <v>59.05</v>
@@ -5691,16 +5691,16 @@
         <v>1881.3</v>
       </c>
       <c r="Q56" s="7" t="n">
-        <v>43</v>
+        <v>42.7</v>
       </c>
       <c r="R56" s="7" t="n">
-        <v>88</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="S56" s="7" t="n">
-        <v>163</v>
+        <v>-20.4</v>
       </c>
       <c r="T56" s="7" t="n">
-        <v>233</v>
+        <v>385.2</v>
       </c>
       <c r="U56" s="5" t="inlineStr">
         <is>
@@ -5756,7 +5756,7 @@
         <v>171177.24</v>
       </c>
       <c r="G57" s="11" t="n">
-        <v>437.75</v>
+        <v>436.6</v>
       </c>
       <c r="H57" s="12" t="n">
         <v>10.82</v>
@@ -5786,16 +5786,16 @@
         <v>1868.2</v>
       </c>
       <c r="Q57" s="12" t="n">
-        <v>44</v>
+        <v>0</v>
       </c>
       <c r="R57" s="12" t="n">
-        <v>89</v>
+        <v>0</v>
       </c>
       <c r="S57" s="12" t="n">
-        <v>164</v>
+        <v>0</v>
       </c>
       <c r="T57" s="12" t="n">
-        <v>234</v>
+        <v>0</v>
       </c>
       <c r="U57" s="10" t="inlineStr">
         <is>
@@ -5851,7 +5851,7 @@
         <v>169609.89</v>
       </c>
       <c r="G58" s="6" t="n">
-        <v>160.7</v>
+        <v>163.85</v>
       </c>
       <c r="H58" s="7" t="n">
         <v>37.12</v>
@@ -5881,16 +5881,16 @@
         <v>987.2</v>
       </c>
       <c r="Q58" s="7" t="n">
-        <v>-10</v>
+        <v>55.5</v>
       </c>
       <c r="R58" s="7" t="n">
-        <v>90</v>
+        <v>167.3</v>
       </c>
       <c r="S58" s="7" t="n">
-        <v>165</v>
+        <v>168.4</v>
       </c>
       <c r="T58" s="7" t="n">
-        <v>235</v>
+        <v>467.9</v>
       </c>
       <c r="U58" s="5" t="inlineStr">
         <is>
@@ -5946,7 +5946,7 @@
         <v>168791.51</v>
       </c>
       <c r="G59" s="11" t="n">
-        <v>681.9</v>
+        <v>675.1</v>
       </c>
       <c r="H59" s="12" t="n">
         <v>39.23</v>
@@ -5976,16 +5976,16 @@
         <v>256</v>
       </c>
       <c r="Q59" s="12" t="n">
-        <v>-9</v>
+        <v>-10.7</v>
       </c>
       <c r="R59" s="12" t="n">
-        <v>91</v>
+        <v>19.8</v>
       </c>
       <c r="S59" s="12" t="n">
-        <v>166</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="T59" s="12" t="n">
-        <v>236</v>
+        <v>326.5</v>
       </c>
       <c r="U59" s="10" t="inlineStr">
         <is>
@@ -6041,7 +6041,7 @@
         <v>168741.33</v>
       </c>
       <c r="G60" s="6" t="n">
-        <v>458.2</v>
+        <v>456.05</v>
       </c>
       <c r="H60" s="7" t="n">
         <v>22.72</v>
@@ -6071,16 +6071,16 @@
         <v>982.1</v>
       </c>
       <c r="Q60" s="7" t="n">
-        <v>-8</v>
+        <v>0</v>
       </c>
       <c r="R60" s="7" t="n">
-        <v>92</v>
+        <v>0</v>
       </c>
       <c r="S60" s="7" t="n">
-        <v>167</v>
+        <v>0</v>
       </c>
       <c r="T60" s="7" t="n">
-        <v>237</v>
+        <v>0</v>
       </c>
       <c r="U60" s="5" t="inlineStr">
         <is>
@@ -6136,7 +6136,7 @@
         <v>165863.5</v>
       </c>
       <c r="G61" s="11" t="n">
-        <v>1629.5</v>
+        <v>1593</v>
       </c>
       <c r="H61" s="12" t="n">
         <v>62.62</v>
@@ -6166,16 +6166,16 @@
         <v>241.5</v>
       </c>
       <c r="Q61" s="12" t="n">
-        <v>-7</v>
+        <v>10.3</v>
       </c>
       <c r="R61" s="12" t="n">
-        <v>93</v>
+        <v>29.6</v>
       </c>
       <c r="S61" s="12" t="n">
-        <v>168</v>
+        <v>37.7</v>
       </c>
       <c r="T61" s="12" t="n">
-        <v>238</v>
+        <v>102.9</v>
       </c>
       <c r="U61" s="10" t="inlineStr">
         <is>
@@ -6231,7 +6231,7 @@
         <v>162731.24</v>
       </c>
       <c r="G62" s="6" t="n">
-        <v>15.02</v>
+        <v>15.42</v>
       </c>
       <c r="H62" s="7" t="n">
         <v>0</v>
@@ -6261,16 +6261,16 @@
         <v>598.3</v>
       </c>
       <c r="Q62" s="7" t="n">
-        <v>-6</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="R62" s="7" t="n">
-        <v>94</v>
+        <v>30.1</v>
       </c>
       <c r="S62" s="7" t="n">
-        <v>169</v>
+        <v>61.5</v>
       </c>
       <c r="T62" s="7" t="n">
-        <v>239</v>
+        <v>76.2</v>
       </c>
       <c r="U62" s="5" t="inlineStr">
         <is>
@@ -6326,7 +6326,7 @@
         <v>159203.81</v>
       </c>
       <c r="G63" s="11" t="n">
-        <v>375.05</v>
+        <v>368.05</v>
       </c>
       <c r="H63" s="12" t="n">
         <v>29.29</v>
@@ -6356,16 +6356,16 @@
         <v>238.5</v>
       </c>
       <c r="Q63" s="12" t="n">
-        <v>-5</v>
+        <v>0</v>
       </c>
       <c r="R63" s="12" t="n">
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="S63" s="12" t="n">
-        <v>170</v>
+        <v>0</v>
       </c>
       <c r="T63" s="12" t="n">
-        <v>240</v>
+        <v>12.2</v>
       </c>
       <c r="U63" s="10" t="inlineStr">
         <is>
@@ -6421,7 +6421,7 @@
         <v>158145.24</v>
       </c>
       <c r="G64" s="6" t="n">
-        <v>239.5</v>
+        <v>233.15</v>
       </c>
       <c r="H64" s="7" t="n">
         <v>76.53</v>
@@ -6451,16 +6451,16 @@
         <v>237</v>
       </c>
       <c r="Q64" s="7" t="n">
-        <v>-4</v>
+        <v>-24</v>
       </c>
       <c r="R64" s="7" t="n">
-        <v>96</v>
+        <v>6.5</v>
       </c>
       <c r="S64" s="7" t="n">
-        <v>171</v>
+        <v>0</v>
       </c>
       <c r="T64" s="7" t="n">
-        <v>241</v>
+        <v>0.8</v>
       </c>
       <c r="U64" s="5" t="inlineStr">
         <is>
@@ -6516,7 +6516,7 @@
         <v>157062.74</v>
       </c>
       <c r="G65" s="11" t="n">
-        <v>1839</v>
+        <v>1823.4</v>
       </c>
       <c r="H65" s="12" t="n">
         <v>27.31</v>
@@ -6546,16 +6546,16 @@
         <v>228.4</v>
       </c>
       <c r="Q65" s="12" t="n">
-        <v>-3</v>
+        <v>7.5</v>
       </c>
       <c r="R65" s="12" t="n">
-        <v>97</v>
+        <v>60.3</v>
       </c>
       <c r="S65" s="12" t="n">
-        <v>172</v>
+        <v>196.6</v>
       </c>
       <c r="T65" s="12" t="n">
-        <v>242</v>
+        <v>567.3</v>
       </c>
       <c r="U65" s="10" t="inlineStr">
         <is>
@@ -6611,7 +6611,7 @@
         <v>157024.11</v>
       </c>
       <c r="G66" s="6" t="n">
-        <v>7410</v>
+        <v>7387</v>
       </c>
       <c r="H66" s="7" t="n">
         <v>101.88</v>
@@ -6641,16 +6641,16 @@
         <v>230.8</v>
       </c>
       <c r="Q66" s="7" t="n">
-        <v>-2</v>
+        <v>41.5</v>
       </c>
       <c r="R66" s="7" t="n">
-        <v>98</v>
+        <v>79.8</v>
       </c>
       <c r="S66" s="7" t="n">
-        <v>173</v>
+        <v>248.5</v>
       </c>
       <c r="T66" s="7" t="n">
-        <v>243</v>
+        <v>726.6</v>
       </c>
       <c r="U66" s="5" t="inlineStr">
         <is>
@@ -6706,7 +6706,7 @@
         <v>156517.56</v>
       </c>
       <c r="G67" s="11" t="n">
-        <v>1596.9</v>
+        <v>1559</v>
       </c>
       <c r="H67" s="12" t="n">
         <v>29.42</v>
@@ -6736,16 +6736,16 @@
         <v>587.3</v>
       </c>
       <c r="Q67" s="12" t="n">
-        <v>-1</v>
+        <v>9.4</v>
       </c>
       <c r="R67" s="12" t="n">
-        <v>99</v>
+        <v>37.6</v>
       </c>
       <c r="S67" s="12" t="n">
-        <v>174</v>
+        <v>5.5</v>
       </c>
       <c r="T67" s="12" t="n">
-        <v>244</v>
+        <v>91.7</v>
       </c>
       <c r="U67" s="10" t="inlineStr">
         <is>
@@ -6801,7 +6801,7 @@
         <v>152131.18</v>
       </c>
       <c r="G68" s="6" t="n">
-        <v>2853</v>
+        <v>2793.6</v>
       </c>
       <c r="H68" s="7" t="n">
         <v>83.2</v>
@@ -6831,16 +6831,16 @@
         <v>228</v>
       </c>
       <c r="Q68" s="7" t="n">
-        <v>0</v>
+        <v>-40.5</v>
       </c>
       <c r="R68" s="7" t="n">
-        <v>100</v>
+        <v>29.7</v>
       </c>
       <c r="S68" s="7" t="n">
-        <v>175</v>
+        <v>178.5</v>
       </c>
       <c r="T68" s="7" t="n">
-        <v>245</v>
+        <v>323.6</v>
       </c>
       <c r="U68" s="5" t="inlineStr">
         <is>
@@ -6896,7 +6896,7 @@
         <v>150111.75</v>
       </c>
       <c r="G69" s="11" t="n">
-        <v>431.1</v>
+        <v>422.15</v>
       </c>
       <c r="H69" s="12" t="n">
         <v>61.71</v>
@@ -6926,16 +6926,16 @@
         <v>220.5</v>
       </c>
       <c r="Q69" s="12" t="n">
-        <v>1</v>
+        <v>59</v>
       </c>
       <c r="R69" s="12" t="n">
-        <v>101</v>
+        <v>249.3</v>
       </c>
       <c r="S69" s="12" t="n">
-        <v>176</v>
+        <v>518.5</v>
       </c>
       <c r="T69" s="12" t="n">
-        <v>246</v>
+        <v>1407.7</v>
       </c>
       <c r="U69" s="10" t="inlineStr">
         <is>
@@ -6991,7 +6991,7 @@
         <v>146839.26</v>
       </c>
       <c r="G70" s="6" t="n">
-        <v>2970.9</v>
+        <v>3013</v>
       </c>
       <c r="H70" s="7" t="n">
         <v>42.13</v>
@@ -7021,16 +7021,16 @@
         <v>218.3</v>
       </c>
       <c r="Q70" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="R70" s="7" t="n">
-        <v>102</v>
+        <v>0</v>
       </c>
       <c r="S70" s="7" t="n">
-        <v>177</v>
+        <v>0</v>
       </c>
       <c r="T70" s="7" t="n">
-        <v>247</v>
+        <v>0</v>
       </c>
       <c r="U70" s="5" t="inlineStr">
         <is>
@@ -7086,7 +7086,7 @@
         <v>142916.36</v>
       </c>
       <c r="G71" s="11" t="n">
-        <v>187.22</v>
+        <v>183.22</v>
       </c>
       <c r="H71" s="12" t="n">
         <v>6.92</v>
@@ -7116,16 +7116,16 @@
         <v>208.1</v>
       </c>
       <c r="Q71" s="12" t="n">
-        <v>3</v>
+        <v>23.2</v>
       </c>
       <c r="R71" s="12" t="n">
-        <v>103</v>
+        <v>80.3</v>
       </c>
       <c r="S71" s="12" t="n">
-        <v>178</v>
+        <v>297</v>
       </c>
       <c r="T71" s="12" t="n">
-        <v>248</v>
+        <v>661.8</v>
       </c>
       <c r="U71" s="10" t="inlineStr">
         <is>
@@ -7181,7 +7181,7 @@
         <v>141629.12</v>
       </c>
       <c r="G72" s="6" t="n">
-        <v>3977</v>
+        <v>3951.3</v>
       </c>
       <c r="H72" s="7" t="n">
         <v>94.20999999999999</v>
@@ -7211,16 +7211,16 @@
         <v>208</v>
       </c>
       <c r="Q72" s="7" t="n">
-        <v>4</v>
+        <v>27.6</v>
       </c>
       <c r="R72" s="7" t="n">
-        <v>104</v>
+        <v>102.1</v>
       </c>
       <c r="S72" s="7" t="n">
-        <v>179</v>
+        <v>207.8</v>
       </c>
       <c r="T72" s="7" t="n">
-        <v>249</v>
+        <v>431</v>
       </c>
       <c r="U72" s="5" t="inlineStr">
         <is>
@@ -7276,7 +7276,7 @@
         <v>141071.54</v>
       </c>
       <c r="G73" s="11" t="n">
-        <v>31650</v>
+        <v>31135</v>
       </c>
       <c r="H73" s="12" t="n">
         <v>118.43</v>
@@ -7306,16 +7306,16 @@
         <v>1555.3</v>
       </c>
       <c r="Q73" s="12" t="n">
-        <v>5</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="R73" s="12" t="n">
-        <v>105</v>
+        <v>651.5</v>
       </c>
       <c r="S73" s="12" t="n">
-        <v>180</v>
+        <v>1307.2</v>
       </c>
       <c r="T73" s="12" t="n">
-        <v>250</v>
+        <v>3128.8</v>
       </c>
       <c r="U73" s="10" t="inlineStr">
         <is>
@@ -7371,7 +7371,7 @@
         <v>140372.6</v>
       </c>
       <c r="G74" s="6" t="n">
-        <v>891</v>
+        <v>910.7</v>
       </c>
       <c r="H74" s="7" t="n">
         <v>110.3</v>
@@ -7401,16 +7401,16 @@
         <v>1547.9</v>
       </c>
       <c r="Q74" s="7" t="n">
-        <v>6</v>
+        <v>23.6</v>
       </c>
       <c r="R74" s="7" t="n">
-        <v>106</v>
+        <v>133.5</v>
       </c>
       <c r="S74" s="7" t="n">
-        <v>181</v>
+        <v>522.5</v>
       </c>
       <c r="T74" s="7" t="n">
-        <v>251</v>
+        <v>2800.3</v>
       </c>
       <c r="U74" s="5" t="inlineStr">
         <is>
@@ -7466,7 +7466,7 @@
         <v>139570.2</v>
       </c>
       <c r="G75" s="11" t="n">
-        <v>5035</v>
+        <v>5040</v>
       </c>
       <c r="H75" s="12" t="n">
         <v>57.21</v>
@@ -7496,16 +7496,16 @@
         <v>205.1</v>
       </c>
       <c r="Q75" s="12" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="R75" s="12" t="n">
-        <v>107</v>
+        <v>200.6</v>
       </c>
       <c r="S75" s="12" t="n">
-        <v>182</v>
+        <v>462.7</v>
       </c>
       <c r="T75" s="12" t="n">
-        <v>252</v>
+        <v>1061</v>
       </c>
       <c r="U75" s="10" t="inlineStr">
         <is>
@@ -7561,7 +7561,7 @@
         <v>139080.31</v>
       </c>
       <c r="G76" s="6" t="n">
-        <v>3409.8</v>
+        <v>3394</v>
       </c>
       <c r="H76" s="7" t="n">
         <v>49.12</v>
@@ -7591,16 +7591,16 @@
         <v>210.6</v>
       </c>
       <c r="Q76" s="7" t="n">
-        <v>8</v>
+        <v>36.9</v>
       </c>
       <c r="R76" s="7" t="n">
-        <v>108</v>
+        <v>446.5</v>
       </c>
       <c r="S76" s="7" t="n">
-        <v>183</v>
+        <v>2206.8</v>
       </c>
       <c r="T76" s="7" t="n">
-        <v>253</v>
+        <v>6091.5</v>
       </c>
       <c r="U76" s="5" t="inlineStr">
         <is>
@@ -7656,7 +7656,7 @@
         <v>138100.74</v>
       </c>
       <c r="G77" s="11" t="n">
-        <v>46820</v>
+        <v>48785</v>
       </c>
       <c r="H77" s="12" t="n">
         <v>58.44</v>
@@ -7686,16 +7686,16 @@
         <v>803.9</v>
       </c>
       <c r="Q77" s="12" t="n">
-        <v>9</v>
+        <v>31</v>
       </c>
       <c r="R77" s="12" t="n">
-        <v>109</v>
+        <v>150.8</v>
       </c>
       <c r="S77" s="12" t="n">
-        <v>184</v>
+        <v>187.8</v>
       </c>
       <c r="T77" s="12" t="n">
-        <v>254</v>
+        <v>320.2</v>
       </c>
       <c r="U77" s="10" t="inlineStr">
         <is>
@@ -7751,7 +7751,7 @@
         <v>137869.27</v>
       </c>
       <c r="G78" s="6" t="n">
-        <v>407.6</v>
+        <v>405.7</v>
       </c>
       <c r="H78" s="7" t="n">
         <v>40.72</v>
@@ -7781,16 +7781,16 @@
         <v>198.7</v>
       </c>
       <c r="Q78" s="7" t="n">
-        <v>10</v>
+        <v>-13.6</v>
       </c>
       <c r="R78" s="7" t="n">
-        <v>110</v>
+        <v>11.6</v>
       </c>
       <c r="S78" s="7" t="n">
-        <v>185</v>
+        <v>258.2</v>
       </c>
       <c r="T78" s="7" t="n">
-        <v>255</v>
+        <v>596.9</v>
       </c>
       <c r="U78" s="5" t="inlineStr">
         <is>
@@ -7846,7 +7846,7 @@
         <v>136966.62</v>
       </c>
       <c r="G79" s="11" t="n">
-        <v>315.7</v>
+        <v>303.85</v>
       </c>
       <c r="H79" s="12" t="n">
         <v>8.84</v>
@@ -7876,16 +7876,16 @@
         <v>197.3</v>
       </c>
       <c r="Q79" s="12" t="n">
-        <v>11</v>
+        <v>-14.8</v>
       </c>
       <c r="R79" s="12" t="n">
-        <v>111</v>
+        <v>74</v>
       </c>
       <c r="S79" s="12" t="n">
-        <v>186</v>
+        <v>45.5</v>
       </c>
       <c r="T79" s="12" t="n">
-        <v>256</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="U79" s="10" t="inlineStr">
         <is>
@@ -7941,7 +7941,7 @@
         <v>135081.35</v>
       </c>
       <c r="G80" s="6" t="n">
-        <v>4554</v>
+        <v>4430</v>
       </c>
       <c r="H80" s="7" t="n">
         <v>24.08</v>
@@ -7971,16 +7971,16 @@
         <v>202.5</v>
       </c>
       <c r="Q80" s="7" t="n">
-        <v>12</v>
+        <v>-22.1</v>
       </c>
       <c r="R80" s="7" t="n">
-        <v>112</v>
+        <v>-12.5</v>
       </c>
       <c r="S80" s="7" t="n">
-        <v>187</v>
+        <v>-33.7</v>
       </c>
       <c r="T80" s="7" t="n">
-        <v>257</v>
+        <v>51.8</v>
       </c>
       <c r="U80" s="5" t="inlineStr">
         <is>
@@ -8036,7 +8036,7 @@
         <v>134467.44</v>
       </c>
       <c r="G81" s="11" t="n">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H81" s="12" t="n">
         <v>6.09</v>
@@ -8066,16 +8066,16 @@
         <v>195.7</v>
       </c>
       <c r="Q81" s="12" t="n">
-        <v>13</v>
+        <v>-5.6</v>
       </c>
       <c r="R81" s="12" t="n">
-        <v>113</v>
+        <v>58.9</v>
       </c>
       <c r="S81" s="12" t="n">
-        <v>188</v>
+        <v>175.5</v>
       </c>
       <c r="T81" s="12" t="n">
-        <v>258</v>
+        <v>333.6</v>
       </c>
       <c r="U81" s="10" t="inlineStr">
         <is>
@@ -8131,7 +8131,7 @@
         <v>125074.02</v>
       </c>
       <c r="G82" s="6" t="n">
-        <v>8300</v>
+        <v>8373.5</v>
       </c>
       <c r="H82" s="7" t="n">
         <v>43.67</v>
@@ -8161,16 +8161,16 @@
         <v>183.8</v>
       </c>
       <c r="Q82" s="7" t="n">
-        <v>14</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="R82" s="7" t="n">
-        <v>114</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="S82" s="7" t="n">
-        <v>189</v>
+        <v>270.3</v>
       </c>
       <c r="T82" s="7" t="n">
-        <v>259</v>
+        <v>809.5</v>
       </c>
       <c r="U82" s="5" t="inlineStr">
         <is>
@@ -8226,7 +8226,7 @@
         <v>124373.73</v>
       </c>
       <c r="G83" s="11" t="n">
-        <v>8650</v>
+        <v>8837.5</v>
       </c>
       <c r="H83" s="12" t="n">
         <v>59.12</v>
@@ -8256,16 +8256,16 @@
         <v>186.8</v>
       </c>
       <c r="Q83" s="12" t="n">
-        <v>15</v>
+        <v>15.1</v>
       </c>
       <c r="R83" s="12" t="n">
-        <v>35</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="S83" s="12" t="n">
-        <v>190</v>
+        <v>107.4</v>
       </c>
       <c r="T83" s="12" t="n">
-        <v>260</v>
+        <v>317</v>
       </c>
       <c r="U83" s="10" t="inlineStr">
         <is>
@@ -8321,7 +8321,7 @@
         <v>124221.9</v>
       </c>
       <c r="G84" s="6" t="n">
-        <v>11162</v>
+        <v>11046</v>
       </c>
       <c r="H84" s="7" t="n">
         <v>14.03</v>
@@ -8351,16 +8351,16 @@
         <v>182.3</v>
       </c>
       <c r="Q84" s="7" t="n">
-        <v>16</v>
+        <v>-10.2</v>
       </c>
       <c r="R84" s="7" t="n">
-        <v>36</v>
+        <v>59.5</v>
       </c>
       <c r="S84" s="7" t="n">
-        <v>191</v>
+        <v>128.7</v>
       </c>
       <c r="T84" s="7" t="n">
-        <v>261</v>
+        <v>378.9</v>
       </c>
       <c r="U84" s="5" t="inlineStr">
         <is>
@@ -8416,7 +8416,7 @@
         <v>123595.56</v>
       </c>
       <c r="G85" s="11" t="n">
-        <v>239</v>
+        <v>236.6</v>
       </c>
       <c r="H85" s="12" t="n">
         <v>5.6</v>
@@ -8446,16 +8446,16 @@
         <v>179.7</v>
       </c>
       <c r="Q85" s="12" t="n">
-        <v>17</v>
+        <v>-15</v>
       </c>
       <c r="R85" s="12" t="n">
-        <v>37</v>
+        <v>20.6</v>
       </c>
       <c r="S85" s="12" t="n">
-        <v>192</v>
+        <v>142.7</v>
       </c>
       <c r="T85" s="12" t="n">
-        <v>262</v>
+        <v>467.4</v>
       </c>
       <c r="U85" s="10" t="inlineStr">
         <is>
@@ -8511,7 +8511,7 @@
         <v>122878.96</v>
       </c>
       <c r="G86" s="6" t="n">
-        <v>5101.5</v>
+        <v>5064</v>
       </c>
       <c r="H86" s="7" t="n">
         <v>47.19</v>
@@ -8541,16 +8541,16 @@
         <v>177.1</v>
       </c>
       <c r="Q86" s="7" t="n">
-        <v>18</v>
+        <v>-13.2</v>
       </c>
       <c r="R86" s="7" t="n">
-        <v>38</v>
+        <v>14.4</v>
       </c>
       <c r="S86" s="7" t="n">
-        <v>193</v>
+        <v>37.8</v>
       </c>
       <c r="T86" s="7" t="n">
-        <v>263</v>
+        <v>45.8</v>
       </c>
       <c r="U86" s="5" t="inlineStr">
         <is>
@@ -8606,7 +8606,7 @@
         <v>122105.08</v>
       </c>
       <c r="G87" s="11" t="n">
-        <v>1222</v>
+        <v>1212</v>
       </c>
       <c r="H87" s="12" t="n">
         <v>29.6</v>
@@ -8636,16 +8636,16 @@
         <v>183</v>
       </c>
       <c r="Q87" s="12" t="n">
-        <v>19</v>
+        <v>1.2</v>
       </c>
       <c r="R87" s="12" t="n">
-        <v>39</v>
+        <v>53.9</v>
       </c>
       <c r="S87" s="12" t="n">
-        <v>194</v>
+        <v>127.8</v>
       </c>
       <c r="T87" s="12" t="n">
-        <v>264</v>
+        <v>284.1</v>
       </c>
       <c r="U87" s="10" t="inlineStr">
         <is>
@@ -8701,7 +8701,7 @@
         <v>121707.77</v>
       </c>
       <c r="G88" s="6" t="n">
-        <v>194</v>
+        <v>195.24</v>
       </c>
       <c r="H88" s="7" t="n">
         <v>49.89</v>
@@ -8731,16 +8731,16 @@
         <v>180.4</v>
       </c>
       <c r="Q88" s="7" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="R88" s="7" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="S88" s="7" t="n">
-        <v>195</v>
+        <v>0</v>
       </c>
       <c r="T88" s="7" t="n">
-        <v>265</v>
+        <v>0</v>
       </c>
       <c r="U88" s="5" t="inlineStr">
         <is>
@@ -8796,7 +8796,7 @@
         <v>119125.08</v>
       </c>
       <c r="G89" s="11" t="n">
-        <v>684.9</v>
+        <v>695.75</v>
       </c>
       <c r="H89" s="12" t="n">
         <v>180.96</v>
@@ -8826,16 +8826,16 @@
         <v>176.7</v>
       </c>
       <c r="Q89" s="12" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="R89" s="12" t="n">
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="S89" s="12" t="n">
-        <v>196</v>
+        <v>0</v>
       </c>
       <c r="T89" s="12" t="n">
-        <v>266</v>
+        <v>0</v>
       </c>
       <c r="U89" s="10" t="inlineStr">
         <is>
@@ -8891,7 +8891,7 @@
         <v>118840.26</v>
       </c>
       <c r="G90" s="6" t="n">
-        <v>1165</v>
+        <v>1136.3</v>
       </c>
       <c r="H90" s="7" t="n">
         <v>38.49</v>
@@ -8921,16 +8921,16 @@
         <v>1297.1</v>
       </c>
       <c r="Q90" s="7" t="n">
-        <v>22</v>
+        <v>6.5</v>
       </c>
       <c r="R90" s="7" t="n">
-        <v>42</v>
+        <v>79.3</v>
       </c>
       <c r="S90" s="7" t="n">
-        <v>197</v>
+        <v>172.3</v>
       </c>
       <c r="T90" s="7" t="n">
-        <v>267</v>
+        <v>493.4</v>
       </c>
       <c r="U90" s="5" t="inlineStr">
         <is>
@@ -8986,7 +8986,7 @@
         <v>118710.26</v>
       </c>
       <c r="G91" s="11" t="n">
-        <v>546.4</v>
+        <v>533.8</v>
       </c>
       <c r="H91" s="12" t="n">
         <v>60.1</v>
@@ -9016,16 +9016,16 @@
         <v>176</v>
       </c>
       <c r="Q91" s="12" t="n">
-        <v>23</v>
+        <v>-27.1</v>
       </c>
       <c r="R91" s="12" t="n">
-        <v>43</v>
+        <v>-13.7</v>
       </c>
       <c r="S91" s="12" t="n">
-        <v>198</v>
+        <v>-21.6</v>
       </c>
       <c r="T91" s="12" t="n">
-        <v>268</v>
+        <v>-9.5</v>
       </c>
       <c r="U91" s="10" t="inlineStr">
         <is>
@@ -9081,7 +9081,7 @@
         <v>118492.42</v>
       </c>
       <c r="G92" s="6" t="n">
-        <v>879.7</v>
+        <v>859.9</v>
       </c>
       <c r="H92" s="7" t="n">
         <v>9.27</v>
@@ -9111,16 +9111,16 @@
         <v>172.4</v>
       </c>
       <c r="Q92" s="7" t="n">
-        <v>24</v>
+        <v>0.1</v>
       </c>
       <c r="R92" s="7" t="n">
-        <v>44</v>
+        <v>104.7</v>
       </c>
       <c r="S92" s="7" t="n">
-        <v>199</v>
+        <v>399.7</v>
       </c>
       <c r="T92" s="7" t="n">
-        <v>269</v>
+        <v>1385.1</v>
       </c>
       <c r="U92" s="5" t="inlineStr">
         <is>
@@ -9176,7 +9176,7 @@
         <v>117588.5</v>
       </c>
       <c r="G93" s="11" t="n">
-        <v>368</v>
+        <v>365.55</v>
       </c>
       <c r="H93" s="12" t="n">
         <v>30.03</v>
@@ -9206,16 +9206,16 @@
         <v>40012.5</v>
       </c>
       <c r="Q93" s="12" t="n">
-        <v>25</v>
+        <v>-9.699999999999999</v>
       </c>
       <c r="R93" s="12" t="n">
-        <v>45</v>
+        <v>52.7</v>
       </c>
       <c r="S93" s="12" t="n">
-        <v>200</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="T93" s="12" t="n">
-        <v>270</v>
+        <v>601</v>
       </c>
       <c r="U93" s="10" t="inlineStr">
         <is>
@@ -9224,7 +9224,7 @@
       </c>
       <c r="V93" s="10" t="inlineStr">
         <is>
-          <t>Tata Power Renewable Energy Ltd (TPREL) Utility &amp; Group Captive Power Producer</t>
+          <t>Tata Power Renewable Energy Ltd (TPREL) Utility &amp; Group Captive Clean Power Producer</t>
         </is>
       </c>
       <c r="W93" s="10" t="inlineStr">
@@ -9271,7 +9271,7 @@
         <v>117351.62</v>
       </c>
       <c r="G94" s="6" t="n">
-        <v>355.6</v>
+        <v>355.9</v>
       </c>
       <c r="H94" s="7" t="n">
         <v>4.5</v>
@@ -9301,16 +9301,16 @@
         <v>1293.6</v>
       </c>
       <c r="Q94" s="7" t="n">
-        <v>26</v>
+        <v>-11.7</v>
       </c>
       <c r="R94" s="7" t="n">
-        <v>46</v>
+        <v>44.3</v>
       </c>
       <c r="S94" s="7" t="n">
-        <v>201</v>
+        <v>234.2</v>
       </c>
       <c r="T94" s="7" t="n">
-        <v>271</v>
+        <v>410.8</v>
       </c>
       <c r="U94" s="5" t="inlineStr">
         <is>
@@ -9366,7 +9366,7 @@
         <v>116979.88</v>
       </c>
       <c r="G95" s="11" t="n">
-        <v>2913.8</v>
+        <v>2899.7</v>
       </c>
       <c r="H95" s="12" t="n">
         <v>10.29</v>
@@ -9396,16 +9396,16 @@
         <v>170.2</v>
       </c>
       <c r="Q95" s="12" t="n">
-        <v>27</v>
+        <v>-8.800000000000001</v>
       </c>
       <c r="R95" s="12" t="n">
-        <v>47</v>
+        <v>123.3</v>
       </c>
       <c r="S95" s="12" t="n">
-        <v>202</v>
+        <v>97.59999999999999</v>
       </c>
       <c r="T95" s="12" t="n">
-        <v>272</v>
+        <v>135.6</v>
       </c>
       <c r="U95" s="10" t="inlineStr">
         <is>
@@ -9461,7 +9461,7 @@
         <v>114722.07</v>
       </c>
       <c r="G96" s="6" t="n">
-        <v>311.5</v>
+        <v>306.45</v>
       </c>
       <c r="H96" s="7" t="n">
         <v>115.14</v>
@@ -9491,16 +9491,16 @@
         <v>667.8</v>
       </c>
       <c r="Q96" s="7" t="n">
-        <v>28</v>
+        <v>-25.3</v>
       </c>
       <c r="R96" s="7" t="n">
-        <v>48</v>
+        <v>-51.3</v>
       </c>
       <c r="S96" s="7" t="n">
-        <v>203</v>
+        <v>-36.6</v>
       </c>
       <c r="T96" s="7" t="n">
-        <v>273</v>
+        <v>131</v>
       </c>
       <c r="U96" s="5" t="inlineStr">
         <is>
@@ -9556,7 +9556,7 @@
         <v>114490.08</v>
       </c>
       <c r="G97" s="11" t="n">
-        <v>562.1</v>
+        <v>555.7</v>
       </c>
       <c r="H97" s="12" t="n">
         <v>36.95</v>
@@ -9586,16 +9586,16 @@
         <v>170</v>
       </c>
       <c r="Q97" s="12" t="n">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="R97" s="12" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="S97" s="12" t="n">
-        <v>204</v>
+        <v>0</v>
       </c>
       <c r="T97" s="12" t="n">
-        <v>274</v>
+        <v>0</v>
       </c>
       <c r="U97" s="10" t="inlineStr">
         <is>
@@ -9651,7 +9651,7 @@
         <v>114012.23</v>
       </c>
       <c r="G98" s="6" t="n">
-        <v>173.4</v>
+        <v>175.09</v>
       </c>
       <c r="H98" s="7" t="n">
         <v>11.54</v>
@@ -9681,16 +9681,16 @@
         <v>164.2</v>
       </c>
       <c r="Q98" s="7" t="n">
-        <v>30</v>
+        <v>-4.2</v>
       </c>
       <c r="R98" s="7" t="n">
-        <v>50</v>
+        <v>46.5</v>
       </c>
       <c r="S98" s="7" t="n">
-        <v>205</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="T98" s="7" t="n">
-        <v>275</v>
+        <v>209.9</v>
       </c>
       <c r="U98" s="5" t="inlineStr">
         <is>
@@ -9746,7 +9746,7 @@
         <v>113836.67</v>
       </c>
       <c r="G99" s="11" t="n">
-        <v>125.5</v>
+        <v>124.68</v>
       </c>
       <c r="H99" s="12" t="n">
         <v>5.73</v>
@@ -9776,16 +9776,16 @@
         <v>165.6</v>
       </c>
       <c r="Q99" s="12" t="n">
-        <v>31</v>
+        <v>-9</v>
       </c>
       <c r="R99" s="12" t="n">
-        <v>51</v>
+        <v>62.2</v>
       </c>
       <c r="S99" s="12" t="n">
-        <v>206</v>
+        <v>190.6</v>
       </c>
       <c r="T99" s="12" t="n">
-        <v>276</v>
+        <v>623.2</v>
       </c>
       <c r="U99" s="10" t="inlineStr">
         <is>
@@ -9841,7 +9841,7 @@
         <v>111888.39</v>
       </c>
       <c r="G100" s="6" t="n">
-        <v>1385</v>
+        <v>1384</v>
       </c>
       <c r="H100" s="7" t="n">
         <v>31.26</v>
@@ -9871,16 +9871,16 @@
         <v>164.6</v>
       </c>
       <c r="Q100" s="7" t="n">
-        <v>32</v>
+        <v>-7.8</v>
       </c>
       <c r="R100" s="7" t="n">
-        <v>52</v>
+        <v>15.3</v>
       </c>
       <c r="S100" s="7" t="n">
-        <v>207</v>
+        <v>52.9</v>
       </c>
       <c r="T100" s="7" t="n">
-        <v>277</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="U100" s="5" t="inlineStr">
         <is>
@@ -9936,7 +9936,7 @@
         <v>111720.43</v>
       </c>
       <c r="G101" s="11" t="n">
-        <v>1120</v>
+        <v>1145.5</v>
       </c>
       <c r="H101" s="12" t="n">
         <v>22.95</v>
@@ -9966,16 +9966,16 @@
         <v>162.3</v>
       </c>
       <c r="Q101" s="12" t="n">
-        <v>33</v>
+        <v>17.6</v>
       </c>
       <c r="R101" s="12" t="n">
-        <v>53</v>
+        <v>99.7</v>
       </c>
       <c r="S101" s="12" t="n">
-        <v>208</v>
+        <v>127.8</v>
       </c>
       <c r="T101" s="12" t="n">
-        <v>278</v>
+        <v>174.2</v>
       </c>
       <c r="U101" s="10" t="inlineStr">
         <is>
@@ -10031,7 +10031,7 @@
         <v>111366.19</v>
       </c>
       <c r="G102" s="6" t="n">
-        <v>1640.7</v>
+        <v>1672.2</v>
       </c>
       <c r="H102" s="7" t="n">
         <v>61.03</v>
@@ -10061,16 +10061,16 @@
         <v>163.8</v>
       </c>
       <c r="Q102" s="7" t="n">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="R102" s="7" t="n">
-        <v>54</v>
+        <v>0</v>
       </c>
       <c r="S102" s="7" t="n">
-        <v>209</v>
+        <v>0</v>
       </c>
       <c r="T102" s="7" t="n">
-        <v>279</v>
+        <v>0.8</v>
       </c>
       <c r="U102" s="5" t="inlineStr">
         <is>
@@ -10126,7 +10126,7 @@
         <v>110956.47</v>
       </c>
       <c r="G103" s="11" t="n">
-        <v>3115.7</v>
+        <v>3200.1</v>
       </c>
       <c r="H103" s="12" t="n">
         <v>72.69</v>
@@ -10156,16 +10156,16 @@
         <v>163.2</v>
       </c>
       <c r="Q103" s="12" t="n">
-        <v>35</v>
+        <v>0.5</v>
       </c>
       <c r="R103" s="12" t="n">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="S103" s="12" t="n">
-        <v>210</v>
+        <v>0</v>
       </c>
       <c r="T103" s="12" t="n">
-        <v>280</v>
+        <v>-1.2</v>
       </c>
       <c r="U103" s="10" t="inlineStr">
         <is>

</xml_diff>